<commit_message>
Reject non-dict Overpass payloads with a clear actionable error
If a cached file is valid JSON but not an object (e.g. someone manually
edited it down to [], null, or a bare string), the subsequent payload.pop /
payload.get calls would raise an unhelpful AttributeError with no clue
where the bad data came from.

Adds an isinstance(payload, dict) guard that runs after the fetch-or-cache
selection. On failure it raises RuntimeError naming the source (live
response or the exact cache file path) and the actual type/snippet so
the operator can fix the cache file and re-run.

Verified via a temp-cache test that writes "[]" to a fake snapshot and
forces the live query to fail: the function now raises with the file
path in the message instead of an AttributeError from .pop().

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tiger_audit_blue_ash_montgomery/reports/TIGER-Audit-Blue-Ash-Montgomery.xlsx
+++ b/tiger_audit_blue_ash_montgomery/reports/TIGER-Audit-Blue-Ash-Montgomery.xlsx
@@ -561,7 +561,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Audit date (UTC): 2026-04-29T02:42:02+00:00</t>
+          <t>Audit date (UTC): 2026-04-29T02:49:14+00:00</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Woodford Road</t>
+          <t>East Columbia Avenue</t>
         </is>
       </c>
       <c r="C16" s="5" t="n">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>tertiary</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -2154,18 +2154,18 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>East Columbia Avenue</t>
+          <t>Hosbrook Road</t>
         </is>
       </c>
       <c r="C17" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="D17" s="5" t="n">
-        <v>0</v>
+      <c r="D17" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>secondary</t>
+          <t>residential</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -2180,18 +2180,18 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Hosbrook Road</t>
+          <t>Kugler Mill Road</t>
         </is>
       </c>
       <c r="C18" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="D18" s="10" t="n">
-        <v>2</v>
+      <c r="D18" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>residential</t>
+          <t>residential, tertiary, unclassified</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Kugler Mill Road</t>
+          <t>Woodford Road</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>residential, tertiary, unclassified</t>
+          <t>tertiary</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Malsbary Road</t>
+          <t>Fox Run Drive</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
@@ -2347,7 +2347,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>residential</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Fox Run Drive</t>
+          <t>Malsbary Road</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>residential</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -2388,18 +2388,18 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Hunters Creek Drive</t>
+          <t>Miami Road</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="D26" s="10" t="n">
-        <v>2</v>
+      <c r="D26" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>residential, service</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -2440,18 +2440,18 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Miami Road</t>
+          <t>Hunters Creek Drive</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="D28" s="5" t="n">
-        <v>0</v>
+      <c r="D28" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>secondary</t>
+          <t>residential, service</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Alamo Avenue</t>
+          <t>Commons Road</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>tertiary</t>
+          <t>residential</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Commons Road</t>
+          <t>Alamo Avenue</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
@@ -2555,7 +2555,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>residential</t>
+          <t>tertiary</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -73253,7 +73253,7 @@
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>2026-04-29T02:42:02+00:00</t>
+          <t>2026-04-29T02:49:14+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-overlay place labels when imagery basemap is selected
Esri/USGS satellite tiles ship without place names or street labels —
on the combined Hamilton-County view at full zoom-out, the map looked
empty except for the orange defect polylines and purple gap clusters,
with no way to tell which cluster is in which neighborhood.

This adds a transparent CARTO "voyager_only_labels" tile layer that
auto-stacks above any imagery basemap (Esri Imagery / Clarity / USGS
Imagery / Ohio OSIP / Esri Wayback). Each BMS entry that needs labels
now carries `labels: true`; setBasemap reads the flag and adds/removes
the overlay alongside the basemap. CARTO's own basemaps and the
topographic options keep their built-in labels and don't get the
overlay.

Z-order is still correct: the labels live in tilePane, polylines in
overlayPane, gap markers in markerPane — so labels appear above
imagery but below all defect data.
</commit_message>
<xml_diff>
--- a/tiger_audit_blue_ash_montgomery/reports/TIGER-Audit-Blue-Ash-Montgomery.xlsx
+++ b/tiger_audit_blue_ash_montgomery/reports/TIGER-Audit-Blue-Ash-Montgomery.xlsx
@@ -561,7 +561,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Audit date (UTC): 2026-04-29T02:49:14+00:00</t>
+          <t>Audit date (UTC): 2026-04-29T13:07:54+00:00</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>East Columbia Avenue</t>
+          <t>Woodford Road</t>
         </is>
       </c>
       <c r="C16" s="5" t="n">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>secondary</t>
+          <t>tertiary</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Woodford Road</t>
+          <t>East Columbia Avenue</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>tertiary</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -2310,18 +2310,18 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Reed Hartman Highway</t>
+          <t>Malsbary Road</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="D23" s="5" t="n">
-        <v>0</v>
+      <c r="D23" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>secondary</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -2362,18 +2362,18 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Malsbary Road</t>
+          <t>Reed Hartman Highway</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="D25" s="10" t="n">
-        <v>4</v>
+      <c r="D25" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -2388,7 +2388,7 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Miami Road</t>
+          <t>Stewart Avenue</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>secondary</t>
+          <t>residential, secondary, tertiary</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Stewart Avenue</t>
+          <t>Miami Road</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>residential, secondary, tertiary</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Eastwood Drive</t>
+          <t>Alamo Avenue</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>residential</t>
+          <t>tertiary</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Schenck Avenue</t>
+          <t>Dawson Road</t>
         </is>
       </c>
       <c r="C30" s="5" t="n">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>residential</t>
+          <t>tertiary</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Commons Road</t>
+          <t>Eastwood Drive</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Alamo Avenue</t>
+          <t>Laurel Avenue</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
@@ -2555,7 +2555,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>tertiary</t>
+          <t>residential</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -2570,7 +2570,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Dawson Road</t>
+          <t>Commons Road</t>
         </is>
       </c>
       <c r="C33" s="5" t="n">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>tertiary</t>
+          <t>residential</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Laurel Avenue</t>
+          <t>Schenck Avenue</t>
         </is>
       </c>
       <c r="C34" s="5" t="n">
@@ -73253,7 +73253,7 @@
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>2026-04-29T02:49:14+00:00</t>
+          <t>2026-04-29T13:07:54+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add --from-cache, --from-csv, --self-test reproducibility flags
Three new CLI flags for offline reproducibility and self-verification:

- --from-cache: skip Overpass API, use newest cached JSON per zone
- --from-csv: rebuild from previously written CSVs (skip fetch + classify)
- --self-test: compare output counts against all_zones_summary.csv reference

Canonical reproducibility command:
  python tiger_audit.py --zone all --from-cache --self-test

Regenerated outputs reflect the verification run (timestamp-only changes).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tiger_audit_blue_ash_montgomery/reports/TIGER-Audit-Blue-Ash-Montgomery.xlsx
+++ b/tiger_audit_blue_ash_montgomery/reports/TIGER-Audit-Blue-Ash-Montgomery.xlsx
@@ -561,7 +561,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Audit date (UTC): 2026-04-29T13:07:54+00:00</t>
+          <t>Audit date (UTC): 2026-04-30T17:05:33+00:00</t>
         </is>
       </c>
     </row>
@@ -2154,18 +2154,18 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Hosbrook Road</t>
+          <t>East Columbia Avenue</t>
         </is>
       </c>
       <c r="C17" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="D17" s="10" t="n">
-        <v>2</v>
+      <c r="D17" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>residential</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -2206,18 +2206,18 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>East Columbia Avenue</t>
+          <t>Hosbrook Road</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="D19" s="5" t="n">
-        <v>0</v>
+      <c r="D19" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>secondary</t>
+          <t>residential</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -2310,18 +2310,18 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Malsbary Road</t>
+          <t>Reed Hartman Highway</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="D23" s="10" t="n">
-        <v>4</v>
+      <c r="D23" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -2362,18 +2362,18 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Reed Hartman Highway</t>
+          <t>Malsbary Road</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="D25" s="5" t="n">
-        <v>0</v>
+      <c r="D25" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>secondary</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -2388,18 +2388,18 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Stewart Avenue</t>
+          <t>Hunters Creek Drive</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="D26" s="5" t="n">
-        <v>0</v>
+      <c r="D26" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>residential, secondary, tertiary</t>
+          <t>residential, service</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Miami Road</t>
+          <t>Stewart Avenue</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>secondary</t>
+          <t>residential, secondary, tertiary</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -2440,18 +2440,18 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Hunters Creek Drive</t>
+          <t>Miami Road</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="D28" s="10" t="n">
-        <v>2</v>
+      <c r="D28" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>residential, service</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Alamo Avenue</t>
+          <t>Schenck Avenue</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>tertiary</t>
+          <t>residential</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Dawson Road</t>
+          <t>Laurel Avenue</t>
         </is>
       </c>
       <c r="C30" s="5" t="n">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>tertiary</t>
+          <t>residential</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Eastwood Drive</t>
+          <t>Alamo Avenue</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>residential</t>
+          <t>tertiary</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Laurel Avenue</t>
+          <t>Eastwood Drive</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Schenck Avenue</t>
+          <t>Dawson Road</t>
         </is>
       </c>
       <c r="C34" s="5" t="n">
@@ -2607,7 +2607,7 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>residential</t>
+          <t>tertiary</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -73253,7 +73253,7 @@
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>2026-04-29T13:07:54+00:00</t>
+          <t>2026-04-30T17:05:33+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>